<commit_message>
Backend y frontend parte 1. gestion usuarios, seguridad avanzada
</commit_message>
<xml_diff>
--- a/plantilla_requisitos.xlsx
+++ b/plantilla_requisitos.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROGRAMACION\SG_Regional_Conquis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3D4CFEB-0399-41E0-8A81-5EB7E1E9B1E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29549E1-1A73-4DC7-9C77-0ABDC910EF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{454A58D9-111B-4B1E-8F30-788A9DDFA1AD}"/>
   </bookViews>
@@ -451,6 +451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DBBD629-8FCE-425A-98A5-287F429D24B0}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -532,11 +533,11 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo de Condicion de la clase" prompt="&gt;&gt;Si son clases de conquistadores Elegir Regular o Avanzada segun corresponda_x000a_&gt;&gt;Si son ConquisMas elegir Nivel 1 o 2 segun corresponda" sqref="B2:B4" xr:uid="{DCBAF5B8-B47F-404C-9629-DDCD59974D15}">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Tipo de Condicion de la clase" prompt="&gt;&gt;Si son clases de conquistadores Elegir Regular o Avanzada segun corresponda_x000a_&gt;&gt;Si son ConquisMas elegir Nivel 1 o 2 segun corresponda" sqref="B3:B4 B2" xr:uid="{DCBAF5B8-B47F-404C-9629-DDCD59974D15}">
       <formula1>"Regular, Avanzada, Nivel 1, Nivel 2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C4" xr:uid="{979FDB0E-5BC2-4B24-A1F7-A801604E6F7F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C3" xr:uid="{979FDB0E-5BC2-4B24-A1F7-A801604E6F7F}">
       <formula1>"I, II, III, IV, V, VI, VII, VII, IX, AV"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A4" xr:uid="{C74E8162-B4F0-4336-8836-64D6DA733ECD}">
@@ -547,6 +548,9 @@
       <formula2>15</formula2>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Requisito" prompt="Colocar descripcion del requisito " sqref="E2:E4" xr:uid="{9D783569-755B-444C-AD86-24A0E165CCE4}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C4" xr:uid="{1D9F266D-6AA6-4EC8-9C34-6DF0745C1FF8}">
+      <formula1>"I, II, III, IV, V, VI, VII, VII, IX, AV, C+Gen, C+GM, C+AG, C+CA"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>